<commit_message>
this version almost fix everything one step left
</commit_message>
<xml_diff>
--- a/model/Tous_les_Emplois_du_Temps.xlsx
+++ b/model/Tous_les_Emplois_du_Temps.xlsx
@@ -94,14 +94,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6E0B4"/>
-        <bgColor rgb="00C6E0B4"/>
+        <fgColor rgb="00B4C7E7"/>
+        <bgColor rgb="00B4C7E7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B4C7E7"/>
-        <bgColor rgb="00B4C7E7"/>
+        <fgColor rgb="00C6E0B4"/>
+        <bgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
   </fills>
@@ -137,13 +137,13 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -584,24 +584,134 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
+          <t>[SYR210] Systèmes Logiques
+(CM Online)
+Prof: Yehjebouha
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(TD)
+Prof: Meya
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Sidi Soueina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
           <t>[MAI210] Algèbre II
 (CM)
 Prof: Tah
 Salle: 101</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI2
+Prof: Med Lemine
+Salle: En ligne /// [RSS210] Services Reseaux
+(TP) - RSS-TP1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
 (TP) - TD1
-Prof: Sidi Mouhamed
+Prof: Debagh
 Salle: 102 /// [DEV210] Programmation Python
 (TP) - TD2
 Prof: Esseyssah
 Salle: 103</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -609,29 +719,82 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(TP) - TD1
+Prof: Kaber
+Salle: 102 /// [DEV211] Langages Web
+(TP) - TD2
+Prof: Aicha
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(TD)
+Prof: Yehjebouha
 Salle: 101</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI1
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TP1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TP2
+Prof: Esseyssah
+Salle: 103 /// [CNM210] CMS et PAO
+(TD Online) - DWM
+Prof: Cheikhani
+Salle: En ligne /// [RSS210] Services Reseaux
+(TD Online) - RSS
+Prof: Saw
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Debagh
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI2
@@ -642,132 +805,35 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
 Salle: 101</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(TP) - TD1
-Prof: Debagh
-Salle: 102 /// [DEV211] Langages Web
-(TP) - TD2
-Prof: Aicha
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
 Salle: 101</t>
         </is>
       </c>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Sidi Soueina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Hassina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP) - DSI1-TD1
-Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI1-TD2
-Prof: Esseyssah
-Salle: 103 /// [CNM210] CMS et PAO
-(TD Online) - DWM
-Prof: Cheikhani
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Debagh
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
@@ -775,48 +841,10 @@
 Salle: 101 /// [CNM210] CMS et PAO
 (CM) - DWM
 Prof: Cheikhani
-Salle: 201 /// [RSS210] Services Reseaux
-(TP) - RSS-TD1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TD2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD1
-Prof: Kaber
-Salle: 102 /// [SYR211] Systèmes d’exploitation
-(TP) - TD2
-Prof: Debagh
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>[MAI211] Probabilités et Statistiques
 (CM)
@@ -824,26 +852,26 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
-(TP) - DSI2-TD1
+(TP Online) - DSI2-TP1
 Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI2-TD2
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
 Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
 Salle: 101</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -851,7 +879,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -939,13 +967,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -957,13 +985,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -975,13 +1003,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -993,13 +1021,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1011,13 +1039,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1105,13 +1133,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1123,13 +1151,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1141,13 +1169,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1159,13 +1187,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1177,13 +1205,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1271,13 +1299,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1289,13 +1317,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1307,13 +1335,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1325,13 +1353,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1343,13 +1371,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1437,13 +1465,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1455,13 +1483,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1473,13 +1501,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1491,13 +1519,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1509,13 +1537,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1603,13 +1631,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1621,13 +1649,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1639,13 +1667,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1657,13 +1685,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1675,13 +1703,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1769,13 +1797,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1787,13 +1815,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1805,13 +1833,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1823,13 +1851,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1841,13 +1869,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1935,13 +1963,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1953,13 +1981,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1971,13 +1999,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1989,13 +2017,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2007,13 +2035,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2101,13 +2129,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2119,13 +2147,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2137,13 +2165,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2155,13 +2183,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2173,13 +2201,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2267,13 +2295,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2285,13 +2313,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2303,13 +2331,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2321,21 +2349,43 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
-(TP) - DSI1-TD1
+(CM Online)
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TP1
 Prof: Med Lemine
 Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI1-TD2
+(TP) - DSI1-TP2
 Prof: Esseyssah
 Salle: 103</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM)
@@ -2343,26 +2393,11 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2450,13 +2485,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2468,13 +2503,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2486,13 +2521,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2504,13 +2539,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2522,13 +2557,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2616,8 +2651,7 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
@@ -2625,7 +2659,34 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(TP) - TD3
+Prof: Sidi Mouhamed
+Salle: 102 /// [DEV210] Programmation Python
+(TP) - TD4
+Prof: Esseyssah
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM Online)
+Prof: Yehjebouha
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
@@ -2633,7 +2694,93 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Sidi Soueina
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI2
+Prof: Med Lemine
+Salle: En ligne /// [RSS210] Services Reseaux
+(TP) - RSS-TP1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Debagh
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (CM)
@@ -2641,7 +2788,24 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Bekar
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -2649,20 +2813,61 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI1
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TP1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TP2
+Prof: Esseyssah
+Salle: 103 /// [CNM210] CMS et PAO
+(TD Online) - DWM
+Prof: Cheikhani
+Salle: En ligne /// [RSS210] Services Reseaux
+(TD Online) - RSS
+Prof: Saw
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI2
@@ -2673,157 +2878,18 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Sidi Soueina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Hassina
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Debagh
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (TP) - TD3
 Prof: Kaber
-Salle: 102 /// [DEV210] Programmation Python
+Salle: 102 /// [SYR211] Systèmes d’exploitation
 (TP) - TD4
-Prof: Esseyssah
+Prof: Debagh
 Salle: 103</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Bekar
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP) - DSI1-TD1
-Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI1-TD2
-Prof: Esseyssah
-Salle: 103 /// [CNM210] CMS et PAO
-(TD Online) - DWM
-Prof: Cheikhani
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM) - DSI1
-Prof: Med Lemine
-Salle: 101 /// [CNM210] CMS et PAO
-(CM) - DWM
-Prof: Cheikhani
-Salle: 201 /// [RSS210] Services Reseaux
-(TP) - RSS-TD1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TD2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2835,7 +2901,7 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (TP) - TD3
@@ -2846,8 +2912,18 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM) - DSI1
+Prof: Med Lemine
+Salle: 101 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -2855,27 +2931,34 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
-(TP) - DSI2-TD1
+(TP Online) - DSI2-TP1
 Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI2-TD2
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
 Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(TD)
+Prof: Meya
 Salle: 201</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(TD)
+Prof: Yehjebouha
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2963,13 +3046,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2981,7 +3064,64 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(TP) - RSS-TP1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(TD Online)
+Prof: Saw
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>[RSS210] Services Reseaux
 (CM)
@@ -2989,58 +3129,8 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>[RSS210] Services Reseaux
-(TP) - RSS-TD1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TD2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3052,13 +3142,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3146,13 +3236,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3164,13 +3254,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3182,13 +3272,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3200,13 +3290,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3218,13 +3308,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3312,13 +3402,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3330,13 +3420,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3348,13 +3438,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3366,9 +3456,9 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>[CNM210] CMS et PAO
 (TD Online)
@@ -3376,8 +3466,23 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>[CNM210] CMS et PAO
 (CM)
@@ -3385,26 +3490,11 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3492,13 +3582,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3513,53 +3603,60 @@
       <c r="B4" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
+(CM Online)
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
 (CM)
 Prof: Med Lemine
 Salle: 201</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3571,23 +3668,23 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
-(TP) - DSI2-TD1
+(TP Online) - DSI2-TP1
 Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI2-TD2
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
 Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3675,13 +3772,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3693,13 +3790,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3711,13 +3808,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3729,13 +3826,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3747,13 +3844,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3841,15 +3938,15 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
 Salle: 201</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (TP) - TD5
@@ -3860,7 +3957,7 @@
 Salle: 204</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (TP) - TD5
@@ -3871,7 +3968,73 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Cheiba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI2
+Prof: Med Lemine
+Salle: En ligne /// [RSS210] Services Reseaux
+(TP) - RSS-TP1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
@@ -3879,7 +4042,60 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Meya
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(TP) - TD6
+Prof: Mahfoudh
+Salle: 102</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(TD)
+Prof: Hassina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (CM)
@@ -3887,27 +4103,61 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
 Prof: Moussa
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI1
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TP1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TP2
+Prof: Esseyssah
+Salle: 103 /// [CNM210] CMS et PAO
+(TD Online) - DWM
+Prof: Cheikhani
+Salle: En ligne /// [RSS210] Services Reseaux
+(TD Online) - RSS
+Prof: Saw
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI2
@@ -3918,64 +4168,27 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Meya
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Sidi Mouhamed
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Cheiba
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM Online)
+Prof: Marba
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -3983,57 +4196,7 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP) - DSI1-TD1
-Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI1-TD2
-Prof: Esseyssah
-Salle: 103 /// [CNM210] CMS et PAO
-(TD Online) - DWM
-Prof: Cheikhani
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(TP) - TD6
-Prof: Mahfoudh
-Salle: 102</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
@@ -4041,57 +4204,10 @@
 Salle: 101 /// [CNM210] CMS et PAO
 (CM) - DWM
 Prof: Cheikhani
-Salle: 201 /// [RSS210] Services Reseaux
-(TP) - RSS-TD1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TD2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
 Salle: 201</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP) - DSI2-TD1
-Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI2-TD2
-Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (CM)
@@ -4099,15 +4215,34 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP1
+Prof: Med Lemine
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
+Prof: Esseyssah
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(TD)
+Prof: Marba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>[SPEC211] PI 1
 (CM)
 Prof: Encadreur
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4195,7 +4330,7 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -4206,12 +4341,12 @@
       <c r="C3" s="7" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
-(CM Online)
+(TD)
 Prof: Marba
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>[DPR212] Projet Personnel et Professionnel II
 (CM)
@@ -4219,7 +4354,7 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (TP) - TD7
@@ -4230,23 +4365,23 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
 Prof: Lam
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4258,7 +4393,163 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI2
+Prof: Med Lemine
+Salle: En ligne /// [RSS210] Services Reseaux
+(TP) - RSS-TP1
+Prof: Souvi
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM Online)
+Prof: Marba
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(TP) - TD7
+Prof: Meya
+Salle: 102 /// [DEV211] Langages Web
+(TP) - TD8
+Prof: Aicha
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Cheiba
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(TD)
+Prof: Hassina
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI1
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(TP) - DSI1-TP1
+Prof: Med Lemine
+Salle: 102 /// [DSI210] Systeme de getion de BD
+(TP) - DSI1-TP2
+Prof: Esseyssah
+Salle: 103 /// [CNM210] CMS et PAO
+(TD Online) - DWM
+Prof: Cheikhani
+Salle: En ligne /// [RSS210] Services Reseaux
+(TD Online) - RSS
+Prof: Saw
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI2
@@ -4269,124 +4560,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Sidi Mouhamed
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Cheiba
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(TP) - TD8
-Prof: Mahfoudh
-Salle: 102</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 203</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(TP) - TD7
-Prof: Meya
-Salle: 102 /// [DEV211] Langages Web
-(TP) - TD8
-Prof: Aicha
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP) - DSI1-TD1
-Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI1-TD2
-Prof: Esseyssah
-Salle: 103 /// [CNM210] CMS et PAO
-(TD Online) - DWM
-Prof: Cheikhani
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -4394,7 +4568,27 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Marba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
@@ -4402,73 +4596,38 @@
 Salle: 101 /// [CNM210] CMS et PAO
 (CM) - DWM
 Prof: Cheikhani
-Salle: 201 /// [RSS210] Services Reseaux
-(TP) - RSS-TD1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TD2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
 Prof: Habeb
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(TD)
-Prof: Marba
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
-(TP) - DSI2-TD1
+(TP Online) - DSI2-TP1
 Prof: Med Lemine
-Salle: 102 /// [DSI210] Systeme de getion de BD
-(TP) - DSI2-TD2
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
 Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr">
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>[MAI212] Préparation à la certification PIX 2
 (CM)
 Prof: Meya
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4556,13 +4715,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4574,13 +4733,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4592,13 +4751,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4610,13 +4769,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4628,13 +4787,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4722,13 +4881,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4740,13 +4899,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4758,13 +4917,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4776,13 +4935,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4794,13 +4953,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4888,13 +5047,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4906,13 +5065,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4924,13 +5083,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4942,13 +5101,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4960,13 +5119,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5054,13 +5213,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5072,13 +5231,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5090,13 +5249,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5108,13 +5267,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5126,13 +5285,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5220,13 +5379,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
-      <c r="E3" s="7" t="inlineStr"/>
-      <c r="F3" s="7" t="inlineStr"/>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="inlineStr"/>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5238,13 +5397,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="7" t="inlineStr"/>
-      <c r="G4" s="7" t="inlineStr"/>
-      <c r="H4" s="7" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5256,13 +5415,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr"/>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr"/>
+      <c r="C5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5274,13 +5433,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="7" t="inlineStr"/>
-      <c r="G6" s="7" t="inlineStr"/>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5292,13 +5451,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr"/>
+      <c r="C7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>x</t>
         </is>

</xml_diff>

<commit_message>
Fixed the website now everything is perfect we can publish it and it would work perfectly as the university official website. except for the groups of type language & ppp i still haven't tested it
</commit_message>
<xml_diff>
--- a/model/Tous_les_Emplois_du_Temps.xlsx
+++ b/model/Tous_les_Emplois_du_Temps.xlsx
@@ -94,14 +94,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B4C7E7"/>
-        <bgColor rgb="00B4C7E7"/>
+        <fgColor rgb="00C6E0B4"/>
+        <bgColor rgb="00C6E0B4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6E0B4"/>
-        <bgColor rgb="00C6E0B4"/>
+        <fgColor rgb="00B4C7E7"/>
+        <bgColor rgb="00B4C7E7"/>
       </patternFill>
     </fill>
   </fills>
@@ -137,13 +137,13 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -585,12 +585,84 @@
       <c r="B3" s="5" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(TP) - TD1
+Prof: Sidi Mouhamed
+Salle: 102 /// [DEV210] Programmation Python
+(TP) - TD2
+Prof: Esseyssah
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
 (CM Online)
 Prof: Yehjebouha
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(TP) - TD1
+Prof: Kaber
+Salle: 102 /// [SYR211] Systèmes d’exploitation
+(TP) - TD2
+Prof: Debagh
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Dyenabe
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(CM) - RSS
+Prof: Souvi
+Salle: 101 /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP1
+Prof: Med Lemine
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
+Prof: Esseyssah
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
@@ -598,7 +670,34 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Sidi Soueina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(TP) - TD1
+Prof: Debagh
+Salle: 102 /// [DEV211] Langages Web
+(TP) - TD2
+Prof: Aicha
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -606,7 +705,51 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Bekar
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>[MAI212] Préparation à la certification PIX 2
 (TD)
@@ -614,141 +757,8 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Sidi Soueina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online) - DSI2
-Prof: Med Lemine
-Salle: En ligne /// [RSS210] Services Reseaux
-(TP) - RSS-TP1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TP2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Hassina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(TP) - TD1
-Prof: Debagh
-Salle: 102 /// [DEV210] Programmation Python
-(TP) - TD2
-Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD1
-Prof: Kaber
-Salle: 102 /// [DEV211] Langages Web
-(TP) - TD2
-Prof: Aicha
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(TD)
-Prof: Yehjebouha
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Dyenabe
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -760,16 +770,9 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online) - DSI1
-Prof: Med Lemine
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (TP) - DSI1-TP1
@@ -786,7 +789,7 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (CM)
@@ -794,18 +797,24 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI2
 Prof: Med Lemine
-Salle: 201 /// [RSS210] Services Reseaux
-(CM) - RSS
+Salle: 201 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 101 /// [RSS210] Services Reseaux
+(TP) - RSS-TP1
 Prof: Souvi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>[SPEC211] PI 1
 (CM)
@@ -813,7 +822,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -825,7 +834,7 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (CM)
@@ -833,45 +842,39 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI2
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
 Prof: Med Lemine
-Salle: 101 /// [CNM210] CMS et PAO
-(CM) - DWM
-Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Bekar
 Salle: 101</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP Online) - DSI2-TP1
-Prof: Med Lemine
-Salle: En ligne /// [DSI210] Systeme de getion de BD
-(TP Online) - DSI2-TP2
-Prof: Esseyssah
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(TD)
+Prof: Yehjebouha
 Salle: 101</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -879,7 +882,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -967,13 +970,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -985,13 +988,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1003,13 +1006,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1021,13 +1024,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1039,13 +1042,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1133,13 +1136,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1151,13 +1154,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1169,13 +1172,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1187,13 +1190,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1205,13 +1208,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1299,13 +1302,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1317,13 +1320,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1335,13 +1338,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1353,13 +1356,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1371,13 +1374,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1465,13 +1468,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1483,13 +1486,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1501,13 +1504,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1519,13 +1522,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1537,13 +1540,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1631,13 +1634,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1649,13 +1652,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1667,13 +1670,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1685,13 +1688,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1703,13 +1706,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1797,13 +1800,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1815,13 +1818,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1833,13 +1836,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1851,13 +1854,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1869,13 +1872,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1963,13 +1966,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1981,13 +1984,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -1999,13 +2002,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2017,13 +2020,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2035,13 +2038,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2129,13 +2132,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2147,13 +2150,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2165,13 +2168,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2183,13 +2186,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2201,13 +2204,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2295,13 +2298,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2313,13 +2316,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2331,13 +2334,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2349,16 +2352,9 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online)
-Prof: Med Lemine
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (TP) - DSI1-TP1
@@ -2369,10 +2365,10 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2384,8 +2380,10 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM)
@@ -2393,11 +2391,9 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2485,13 +2481,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2503,13 +2499,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2521,13 +2517,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2539,13 +2535,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2557,13 +2553,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2651,7 +2647,15 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Tah
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
@@ -2659,26 +2663,15 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(TP) - TD3
-Prof: Sidi Mouhamed
-Salle: 102 /// [DEV210] Programmation Python
-(TP) - TD4
-Prof: Esseyssah
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
 Prof: Dyenabe
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (CM Online)
@@ -2688,13 +2681,99 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Tah
+          <t>[DEV210] Programmation Python
+(TP) - TD4
+Prof: Esseyssah
+Salle: 102</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
 Salle: 201</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(CM) - RSS
+Prof: Souvi
+Salle: 101 /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP1
+Prof: Med Lemine
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
+Prof: Esseyssah
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Sidi Mouhamed
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Yehjebouha
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(TD)
+Prof: Meya
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Hassina
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Debagh
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>[DPR212] Projet Personnel et Professionnel II
 (CM)
@@ -2702,65 +2781,32 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online) - DSI2
-Prof: Med Lemine
-Salle: En ligne /// [RSS210] Services Reseaux
-(TP) - RSS-TP1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TP2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
 Salle: 201</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Sidi Mouhamed
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
 Salle: 201</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Debagh
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Bekar
 Salle: 201</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Hassina
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -2768,44 +2814,20 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Yehjebouha
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Bekar
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hayati
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -2813,43 +2835,7 @@
 Salle: 101</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online) - DSI1
-Prof: Med Lemine
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (TP) - DSI1-TP1
@@ -2866,19 +2852,25 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI2
 Prof: Med Lemine
-Salle: 201 /// [RSS210] Services Reseaux
-(CM) - RSS
+Salle: 201 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 101 /// [RSS210] Services Reseaux
+(TP) - RSS-TP1
 Prof: Souvi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (TP) - TD3
@@ -2889,7 +2881,7 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -2901,7 +2893,7 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (TP) - TD3
@@ -2912,18 +2904,31 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI2
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hayati
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
 Prof: Med Lemine
-Salle: 101 /// [CNM210] CMS et PAO
-(CM) - DWM
-Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -2931,26 +2936,7 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP Online) - DSI2-TP1
-Prof: Med Lemine
-Salle: En ligne /// [DSI210] Systeme de getion de BD
-(TP Online) - DSI2-TP2
-Prof: Esseyssah
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(TD)
-Prof: Meya
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (TD)
@@ -2958,7 +2944,7 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3046,13 +3032,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3064,7 +3050,61 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(CM)
+Prof: Souvi
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(TD Online)
+Prof: Saw
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>[RSS210] Services Reseaux
 (TP) - RSS-TP1
@@ -3075,62 +3115,8 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>[RSS210] Services Reseaux
-(TD Online)
-Prof: Saw
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>[RSS210] Services Reseaux
-(CM)
-Prof: Souvi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3142,13 +3128,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3236,13 +3222,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3254,13 +3240,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3272,13 +3258,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3290,13 +3276,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3308,13 +3294,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3402,13 +3388,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3420,13 +3406,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3438,13 +3424,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3456,9 +3442,9 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>[CNM210] CMS et PAO
 (TD Online)
@@ -3466,10 +3452,17 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>[CNM210] CMS et PAO
+(CM)
+Prof: Cheikhani
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3481,20 +3474,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>[CNM210] CMS et PAO
-(CM)
-Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3582,13 +3568,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3600,78 +3586,7 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online)
-Prof: Med Lemine
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM)
-Prof: Med Lemine
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="80" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>17:00-18:30</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (TP Online) - DSI2-TP1
@@ -3682,9 +3597,80 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM)
+Prof: Med Lemine
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>17:00-18:30</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online)
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3772,13 +3758,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3790,13 +3776,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3808,13 +3794,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3826,13 +3812,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3844,13 +3830,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3938,7 +3924,39 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM Online)
+Prof: Marba
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>[MAI210] Algèbre II
 (CM)
@@ -3946,200 +3964,161 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>09:45-11:15</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(CM) - RSS
+Prof: Souvi
+Salle: 101 /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP1
+Prof: Med Lemine
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
+Prof: Esseyssah
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(TD)
+Prof: Hassina
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>[DPR211] Anglais II
+(CM)
+Prof: Hatabi
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI212] Préparation à la certification PIX 2
+(CM)
+Prof: Meya
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>11:30-13:00</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Cheiba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(CM)
+Prof: Kaber
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>[DPR210] Communication II
+(CM)
+Prof: Lam
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>15:00-16:30</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>[SYR211] Systèmes d’exploitation
+(TP) - TD5
+Prof: Kaber
+Salle: 102 /// [DEV210] Programmation Python
+(TP) - TD6
+Prof: Mahfoudh
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>[DEV211] Langages Web
 (TP) - TD5
 Prof: Meya
-Salle: 104 /// [DEV211] Langages Web
+Salle: 102 /// [DEV211] Langages Web
 (TP) - TD6
 Prof: Aicha
-Salle: 204</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(TP) - TD5
-Prof: Kaber
-Salle: 102 /// [SYR211] Systèmes d’exploitation
-(TP) - TD6
-Prof: Debagh
 Salle: 103</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Cheiba
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="80" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>09:45-11:15</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online) - DSI2
-Prof: Med Lemine
-Salle: En ligne /// [RSS210] Services Reseaux
-(TP) - RSS-TP1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TP2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Sidi Mouhamed
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>[DPR211] Anglais II
-(CM)
-Prof: Hatabi
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(CM)
-Prof: Meya
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>11:30-13:00</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(TP) - TD6
-Prof: Mahfoudh
-Salle: 102</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>[MAI212] Préparation à la certification PIX 2
-(TD)
-Prof: Hassina
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>[DPR210] Communication II
-(CM)
-Prof: Lam
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>[SYR211] Systèmes d’exploitation
-(CM)
-Prof: Kaber
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="80" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>15:00-16:30</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online) - DSI1
-Prof: Med Lemine
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (TP) - DSI1-TP1
@@ -4156,27 +4135,33 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI2
 Prof: Med Lemine
-Salle: 201 /// [RSS210] Services Reseaux
-(CM) - RSS
+Salle: 201 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 101 /// [RSS210] Services Reseaux
+(TP) - RSS-TP1
 Prof: Souvi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
-(CM Online)
+(TD)
 Prof: Marba
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4188,7 +4173,7 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -4196,45 +4181,32 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI2
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(CM)
+Prof: Marba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
 Prof: Med Lemine
-Salle: 101 /// [CNM210] CMS et PAO
-(CM) - DWM
-Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(CM)
-Prof: Marba
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP Online) - DSI2-TP1
-Prof: Med Lemine
-Salle: En ligne /// [DSI210] Systeme de getion de BD
-(TP Online) - DSI2-TP2
-Prof: Esseyssah
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(TD)
-Prof: Marba
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>[SPEC211] PI 1
 (CM)
@@ -4242,7 +4214,7 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4330,31 +4302,26 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>[DEV210] Programmation Python
-(CM)
-Prof: Moussa
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>[SYR210] Systèmes Logiques
-(TD)
-Prof: Marba
-Salle: 201</t>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(TP) - TD7
+Prof: Meya
+Salle: 104 /// [DEV211] Langages Web
+(TP) - TD8
+Prof: Aicha
+Salle: 204</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>[DPR212] Projet Personnel et Professionnel II
-(CM)
-Prof: Yehjebouha
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (TP) - TD7
@@ -4365,15 +4332,23 @@
 Salle: 103</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>[SPEC211] PI 1
+(CM)
+Prof: Encadreur
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>[SYR211] Systèmes d’exploitation
 (CM)
 Prof: Kaber
-Salle: 203</t>
-        </is>
-      </c>
-      <c r="G3" s="6" t="inlineStr">
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
@@ -4381,7 +4356,7 @@
 Salle: 203</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4393,21 +4368,21 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online) - DSI2
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>[RSS210] Services Reseaux
+(CM) - RSS
+Prof: Souvi
+Salle: 101 /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP1
 Prof: Med Lemine
-Salle: En ligne /// [RSS210] Services Reseaux
-(TP) - RSS-TP1
-Prof: Souvi
-Salle: 102 /// [RSS210] Services Reseaux
-(TP) - RSS-TP2
-Prof: Saw
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
+Salle: En ligne /// [DSI210] Systeme de getion de BD
+(TP Online) - DSI2-TP2
+Prof: Esseyssah
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (CM Online)
@@ -4415,26 +4390,23 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>[DEV211] Langages Web
+(CM)
+Prof: Sidi Mouhamed
 Salle: 203</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(TP) - TD7
-Prof: Meya
-Salle: 102 /// [DEV211] Langages Web
-(TP) - TD8
-Prof: Aicha
-Salle: 103</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>[MAI211] Probabilités et Statistiques
+(CM)
+Prof: Cheiba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
@@ -4442,8 +4414,8 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4455,32 +4427,18 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>[DPR210] Communication II
 (CM)
 Prof: Lam
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>[SPEC211] PI 1
-(CM)
-Prof: Encadreur
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>[MAI211] Probabilités et Statistiques
-(CM)
-Prof: Cheiba
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="7" t="inlineStr">
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>[MAI212] Préparation à la certification PIX 2
 (TD)
@@ -4488,15 +4446,15 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>[DEV211] Langages Web
-(CM)
-Prof: Sidi Mouhamed
-Salle: 203</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>[DEV210] Programmation Python
+(CM)
+Prof: Moussa
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4508,23 +4466,23 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>[DPR212] Projet Personnel et Professionnel II
+(CM)
+Prof: Yehjebouha
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>[DPR211] Anglais II
 (CM)
 Prof: Hatabi
-Salle: 202</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(CM Online) - DSI1
-Prof: Med Lemine
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+Salle: 201</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (TP) - DSI1-TP1
@@ -4541,7 +4499,7 @@
 Salle: En ligne</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
@@ -4549,26 +4507,32 @@
 Salle: 201</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI2
 Prof: Med Lemine
-Salle: 201 /// [RSS210] Services Reseaux
-(CM) - RSS
+Salle: 201 /// [CNM210] CMS et PAO
+(CM) - DWM
+Prof: Cheikhani
+Salle: 101 /// [RSS210] Services Reseaux
+(TP) - RSS-TP1
 Prof: Souvi
-Salle: 101</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
+Salle: 102 /// [RSS210] Services Reseaux
+(TP) - RSS-TP2
+Prof: Saw
+Salle: 103</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>[DEV210] Programmation Python
 (CM)
 Prof: Moussa
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4580,7 +4544,7 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>[SYR210] Systèmes Logiques
 (CM)
@@ -4588,38 +4552,39 @@
 Salle: 202</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>[DSI210] Systeme de getion de BD
+(CM Online) - DSI2
+Prof: Med Lemine
+Salle: En ligne</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>[MAI210] Algèbre II
+(CM)
+Prof: Habeb
+Salle: 203</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>[DSI210] Systeme de getion de BD
 (CM) - DSI1
 Prof: Med Lemine
-Salle: 101 /// [CNM210] CMS et PAO
-(CM) - DWM
-Prof: Cheikhani
-Salle: 201</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>[MAI210] Algèbre II
-(CM)
-Prof: Habeb
-Salle: 203</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>[DSI210] Systeme de getion de BD
-(TP Online) - DSI2-TP1
-Prof: Med Lemine
-Salle: En ligne /// [DSI210] Systeme de getion de BD
-(TP Online) - DSI2-TP2
-Prof: Esseyssah
-Salle: En ligne</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr">
+Salle: 101</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>[SYR210] Systèmes Logiques
+(TD)
+Prof: Marba
+Salle: 202</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>[MAI212] Préparation à la certification PIX 2
 (CM)
@@ -4627,7 +4592,7 @@
 Salle: 203</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4715,13 +4680,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4733,13 +4698,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4751,13 +4716,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4769,13 +4734,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4787,13 +4752,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4881,13 +4846,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4899,13 +4864,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4917,13 +4882,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4935,13 +4900,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -4953,13 +4918,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5047,13 +5012,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5065,13 +5030,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5083,13 +5048,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5101,13 +5066,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5119,13 +5084,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5213,13 +5178,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5231,13 +5196,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5249,13 +5214,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5267,13 +5232,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5285,13 +5250,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5379,13 +5344,13 @@
           <t>08:00-09:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-      <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
+      <c r="E3" s="7" t="inlineStr"/>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="7" t="inlineStr"/>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5397,13 +5362,13 @@
           <t>09:45-11:15</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
+      <c r="E4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr"/>
+      <c r="G4" s="7" t="inlineStr"/>
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5415,13 +5380,13 @@
           <t>11:30-13:00</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
-      <c r="G5" s="5" t="inlineStr"/>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5433,13 +5398,13 @@
           <t>15:00-16:30</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr"/>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr"/>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
+      <c r="E6" s="7" t="inlineStr"/>
+      <c r="F6" s="7" t="inlineStr"/>
+      <c r="G6" s="7" t="inlineStr"/>
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -5451,13 +5416,13 @@
           <t>17:00-18:30</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>x</t>
         </is>

</xml_diff>